<commit_message>
updates test plans + mac build script to prevent hangs
</commit_message>
<xml_diff>
--- a/docs/45drives-storage-wizard-test-plan-linux.xlsx
+++ b/docs/45drives-storage-wizard-test-plan-linux.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -507,15 +507,19 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
+          <t>Edition</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Tester</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
@@ -523,7 +527,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Build / Version</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
@@ -531,7 +535,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>OS Version</t>
+          <t>Build / Version</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
@@ -539,7 +543,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Server(s) Under Test</t>
+          <t>OS Version</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
@@ -547,7 +551,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Network Environment</t>
+          <t>Server(s) Under Test</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
@@ -555,27 +559,27 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Total Tests</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>97</t>
-        </is>
-      </c>
+          <t>Network Environment</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr"/>
+          <t>Total Tests</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
@@ -583,7 +587,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Blocked / Skipped</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
@@ -591,37 +595,35 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Blocked / Skipped</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Overall Result</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Test Count</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>1. Installation &amp; First Launch</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2. Dashboard</t>
+          <t>1. Installation &amp; First Launch</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -631,7 +633,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>3. Menu, Themes &amp; Settings</t>
+          <t>2. Dashboard</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -641,150 +643,160 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>4. Set Up a Single Server - Simple Path</t>
+          <t>3. Menu, Themes &amp; Settings</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>5. Set Up a Single Server - Custom Path</t>
+          <t>4. Set Up a Single Server - Simple Path</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>6. Set Up Multiple Servers (Bulk)</t>
+          <t>5. Set Up a Single Server - Custom Path</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>7. Server Management</t>
+          <t>6. Set Up Multiple Servers (Bulk)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>8. Manage Connections (Saved Credentials)</t>
+          <t>7. Server Management</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>9. Back Up This Computer to the Server</t>
+          <t>8. Manage Connections (Saved Credentials)</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>10. Restore from a Local Backup</t>
+          <t>9. Back Up This Computer to the Server</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>11. Remote Backups - Server to Server (Rsync)</t>
+          <t>10. Restore from a Local Backup</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>12. Remote Backups - ZFS Replication</t>
+          <t>11. Remote Backups - Server to Server (Rsync)</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>13. Cloud Accounts &amp; Server to Cloud Backup</t>
+          <t>12. Remote Backups - ZFS Replication</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>14. Off-Site Backups Over a WireShield Tunnel</t>
+          <t>13. Cloud Accounts &amp; Server to Cloud Backup</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>15. Restore from Remote &amp; Cloud Backups</t>
+          <t>14. Off-Site Backups Over a WireShield Tunnel</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>16. Snapshots - Browse, Restore &amp; Rollback</t>
+          <t>15. Restore from Remote &amp; Cloud Backups</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>17. Automatic Updates</t>
+          <t>16. Snapshots - Browse, Restore &amp; Rollback</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
+          <t>17. Automatic Updates</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
           <t>18. Reliability &amp; Edge Cases</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4101,7 +4113,7 @@
       <c r="C98" s="4" t="inlineStr"/>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Uninstall the app (run this last)</t>
+          <t>Uninstall the app - run this last (Linux)</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
@@ -4133,7 +4145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -4259,87 +4271,87 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>What is deliberately NOT in scope</t>
+          <t>Why rsync and ZFS replication are each tested twice</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - WireShield pairing and tunnel management as features in their own right. They are already tested.</t>
+          <t xml:space="preserve">  Sections 11 and 12 run each task type against a plain LAN address. Section 14 runs the same two task types</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Only the handoff between a backup task and WireShield, and backups run over the tunnel, are covered here.</t>
+          <t xml:space="preserve">  again using a WireShield tunnel address. That second pass is not a repeat: it proves the address handed back</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Exhaustive option-by-option coverage of rsync, cloud, and ZFS replication tasks. These are live and stable.</t>
+          <t xml:space="preserve">  from WireShield is usable and that SSH, routing and transfer all work over the WireGuard interface.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    One working task of each type is enough.</t>
+          <t xml:space="preserve">  Cloud backup is run once only, because it goes directly to the provider and never uses the tunnel.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Cloud provider token expiry and access revocation.</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Saved credentials going stale after 30 days - this cannot be triggered within a test window.</t>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>What is deliberately NOT in scope</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - WireShield pairing and tunnel management as features in their own right. They are already tested.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Severity Definitions</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Only the handoff between a backup task and WireShield, and backups run over the tunnel, are covered here.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Critical - The app crashes, data is lost, or something insecure happens</t>
+          <t xml:space="preserve">  - Exhaustive option-by-option coverage of rsync, cloud, and ZFS replication tasks. These are live and stable.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  High - A feature is completely broken with no way around it</t>
+          <t xml:space="preserve">    One working task of each type is enough.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Medium - A feature is partly broken but there is a workaround</t>
+          <t xml:space="preserve">  - Cloud provider token expiry and access revocation.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Low - Cosmetic or a minor annoyance</t>
+          <t xml:space="preserve">  - Saved credentials going stale after 30 days - this cannot be triggered within a test window.</t>
         </is>
       </c>
     </row>
@@ -4349,95 +4361,133 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Test Environment Prerequisites</t>
+          <t>Severity Definitions</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Two 45Drives servers on the same network. At least one with 6 or more drives so Split Pools can be tested.</t>
+          <t xml:space="preserve">  Critical - The app crashes, data is lost, or something insecure happens</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - A third unconfigured server, or the ability to reset one, for the bulk setup and custom setup runs.</t>
+          <t xml:space="preserve">  High - A feature is completely broken with no way around it</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - One cloud account you sign in to (Dropbox or Google Drive) and one that uses keys (S3, Wasabi, or Backblaze B2).</t>
+          <t xml:space="preserve">  Medium - A feature is partly broken but there is a workaround</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Internet access from both servers so the two can pair over WireShield.</t>
+          <t xml:space="preserve">  Low - Cosmetic or a minor annoyance</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Test files including a large file (1 GB+) and files with spaces and accented characters in their names.</t>
-        </is>
-      </c>
+      <c r="A39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - A build of the app one version behind the latest release, so the update tests have something to find.</t>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Test Environment Prerequisites</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Two 45Drives servers on the same network. At least one with 6 or more drives so Split Pools can be tested.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>Note on the WireShield tunnel tests</t>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A third unconfigured server, or the ability to reset one, for the bulk setup and custom setup runs.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Both servers are on the same network for this test pass, so the tunnel tests exercise the local path only.</t>
+          <t xml:space="preserve">  - One cloud account you sign in to (Dropbox or Google Drive) and one that uses keys (S3, Wasabi, or Backblaze B2).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Confirm traffic really went through the tunnel by checking the connection's sent/received counters</t>
+          <t xml:space="preserve">  - Internet access from both servers so the two can pair over WireShield.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Test files including a large file (1 GB+) and files with spaces and accented characters in their names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - A build of the app one version behind the latest release, so the update tests have something to find.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Note on the WireShield tunnel tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Both servers are on the same network for this test pass, so the tunnel tests exercise the local path only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Confirm traffic really went through the tunnel by checking the connection's sent/received counters</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t xml:space="preserve">  before and after each backup that uses the tunnel address.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t xml:space="preserve">  docs/45Drives_Storage_Wizard_User_Guide.md</t>
         </is>

</xml_diff>